<commit_message>
Excel : filtres automatiques + gel première ligne sur les 2 onglets
</commit_message>
<xml_diff>
--- a/benchmark-cartier.xlsx
+++ b/benchmark-cartier.xlsx
@@ -11,7 +11,10 @@
     <sheet name="Grille de scoring" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Méthodologie" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Réponses complètes'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Grille de scoring'!$A$1:$K$52</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -1818,6 +1821,7 @@
       <c r="K18" s="7" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3330,6 +3334,7 @@
       <c r="K52" s="7" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Data viz : 6 radars par catégorie + heatmap récap + footer MT + logo Excel + sidebar data viz
</commit_message>
<xml_diff>
--- a/benchmark-cartier.xlsx
+++ b/benchmark-cartier.xlsx
@@ -207,6 +207,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3345,118 +3375,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A5:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Benchmark Cartier — Méthodologie</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Plateformes testées</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ChatGPT (GPT-4o) — cutoff juin 2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Perplexity (Sonar) — accès web temps réel</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Claude (Sonnet 4) — cutoff mars 2025</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Date du benchmark : 31 mars 2026</t>
+          <t>ChatGPT (GPT-4o) — cutoff juin 2024</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17 requêtes × 3 plateformes = 51 réponses</t>
+          <t>Perplexity (Sonar) — accès web temps réel</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6 catégories d'intention : découverte, comparaison, validation, process, investissement, substitution</t>
-        </is>
-      </c>
-    </row>
+          <t>Claude (Sonnet 4) — cutoff mars 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Grille de scoring</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Date du benchmark : 31 mars 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Présence (0/1) — la maison est-elle citée ?</t>
+          <t>17 requêtes × 3 plateformes = 51 réponses</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Position (1-5) — rang dans la liste</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Exactitude (0-5) — les faits sont-ils justes ?</t>
-        </is>
-      </c>
-    </row>
+          <t>6 catégories d'intention : découverte, comparaison, validation, process, investissement, substitution</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Narratif (0-5) — le récit de marque passe-t-il ?</t>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Grille de scoring</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Actionnabilité (0-5) — peut-on agir (lien, prix, boutique) ?</t>
+          <t>Présence (0/1) — la maison est-elle citée ?</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Position (1-5) — rang dans la liste</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Exactitude (0-5) — les faits sont-ils justes ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Narratif (0-5) — le récit de marque passe-t-il ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Actionnabilité (0-5) — peut-on agir (lien, prix, boutique) ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Sentiment (-1/+1) — ton cohérent avec le positionnement ?</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>